<commit_message>
Started on LDR code
</commit_message>
<xml_diff>
--- a/docs/ldr/ldr.xlsx
+++ b/docs/ldr/ldr.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dayoung\orange\BOAT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dayoung\orange\BOAT\docs\ldr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FCCA0C3-D378-4D57-B320-13A0DF86FC98}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3473CC-DBB2-46FE-958D-9CD066423128}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{342DDD22-8936-4EEA-9C39-5B30C4FFC4A5}"/>
+    <workbookView xWindow="15555" yWindow="4095" windowWidth="21360" windowHeight="15435" xr2:uid="{342DDD22-8936-4EEA-9C39-5B30C4FFC4A5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Ambient Light</t>
   </si>
@@ -69,6 +69,15 @@
   </si>
   <si>
     <t>`</t>
+  </si>
+  <si>
+    <t>LDR</t>
+  </si>
+  <si>
+    <t>Vout</t>
+  </si>
+  <si>
+    <t>Potentiometer</t>
   </si>
 </sst>
 </file>
@@ -420,13 +429,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28D69271-9600-412A-8F94-B492CA344ED6}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -434,7 +444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -442,7 +452,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -450,7 +460,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -458,7 +468,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -466,12 +476,155 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2000</v>
+      </c>
+      <c r="B12">
+        <v>10000</v>
+      </c>
+      <c r="C12">
+        <v>7500</v>
+      </c>
+      <c r="D12">
+        <v>5000</v>
+      </c>
+      <c r="E12">
+        <v>2500</v>
+      </c>
+      <c r="F12">
+        <f>B12/(A12+B12) * 3.3</f>
+        <v>2.75</v>
+      </c>
+      <c r="G12">
+        <f>C12/(A12+C12) * 3.3</f>
+        <v>2.6052631578947367</v>
+      </c>
+      <c r="H12">
+        <f>D12/(A12+D12) * 3.3</f>
+        <v>2.3571428571428572</v>
+      </c>
+      <c r="I12">
+        <f>E12/(A12+E12) * 3.3</f>
+        <v>1.8333333333333333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>5000</v>
+      </c>
+      <c r="B13">
+        <v>10000</v>
+      </c>
+      <c r="C13">
+        <v>7500</v>
+      </c>
+      <c r="D13">
+        <v>5000</v>
+      </c>
+      <c r="E13">
+        <v>2500</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F13:I15" si="0">B13/(A13+B13) * 3.3</f>
+        <v>2.1999999999999997</v>
+      </c>
+      <c r="G13">
+        <f t="shared" ref="G13:G15" si="1">C13/(A13+C13) * 3.3</f>
+        <v>1.9799999999999998</v>
+      </c>
+      <c r="H13">
+        <f t="shared" ref="H13:H15" si="2">D13/(A13+D13) * 3.3</f>
+        <v>1.65</v>
+      </c>
+      <c r="I13">
+        <f t="shared" ref="I13:I15" si="3">E13/(A13+E13) * 3.3</f>
+        <v>1.0999999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>30000</v>
+      </c>
+      <c r="B14">
+        <v>10000</v>
+      </c>
+      <c r="C14">
+        <v>7500</v>
+      </c>
+      <c r="D14">
+        <v>5000</v>
+      </c>
+      <c r="E14">
+        <v>2500</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="1"/>
+        <v>0.66</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="2"/>
+        <v>0.47142857142857136</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>0.25384615384615383</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>140000</v>
+      </c>
+      <c r="B15">
+        <v>10000</v>
+      </c>
+      <c r="C15">
+        <v>7500</v>
+      </c>
+      <c r="D15">
+        <v>5000</v>
+      </c>
+      <c r="E15">
+        <v>2500</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>0.21999999999999997</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="1"/>
+        <v>0.16779661016949152</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="2"/>
+        <v>0.11379310344827585</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="3"/>
+        <v>5.7894736842105256E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>